<commit_message>
Add DQC_0008 reversed-calculation and DQC_0036 period-of-report rules
</commit_message>
<xml_diff>
--- a/reports/dqc_exceptions_2026q2.xlsx
+++ b/reports/dqc_exceptions_2026q2.xlsx
@@ -11,24 +11,27 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0001" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0004" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0005" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0009" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0013" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0014" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0015" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0091" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0095" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0125" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0194" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0195" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0008" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0009" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0013" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0014" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0015" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0036" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0091" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0095" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0125" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0194" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DQC_0195" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DQC_0001'!$A$2:$M$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DQC_0004'!$A$2:$M$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DQC_0009'!$A$2:$M$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'DQC_0014'!$A$2:$M$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DQC_0015'!$A$2:$M$128</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'DQC_0194'!$A$2:$M$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'DQC_0195'!$A$2:$M$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DQC_0009'!$A$2:$M$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'DQC_0014'!$A$2:$M$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'DQC_0015'!$A$2:$M$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'DQC_0036'!$A$2:$M$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'DQC_0194'!$A$2:$M$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'DQC_0195'!$A$2:$M$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -482,7 +485,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>447 findings in 169 of 7,714 filings</t>
+          <t>451 findings in 173 of 7,714 filings</t>
         </is>
       </c>
     </row>
@@ -579,138 +582,138 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>DQC_0009</t>
+          <t>DQC_0008</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Element A must be &lt;= element B (e.g. shares outstanding &lt;= issued)</t>
+          <t>Reversed calculation relative to the US GAAP taxonomy</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>DQC_0013</t>
+          <t>DQC_0009</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Negative tax-rate reconciliation items when pre-tax income is positive</t>
+          <t>Element A must be &lt;= element B (e.g. shares outstanding &lt;= issued)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>DQC_0014</t>
+          <t>DQC_0013</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Negative values with no dimensions (goodwill, revenue, cost of revenue...)</t>
+          <t>Negative tax-rate reconciliation items when pre-tax income is positive</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>DQC_0015</t>
+          <t>DQC_0014</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Negative values for elements that cannot be negative</t>
+          <t>Negative values with no dimensions (goodwill, revenue, cost of revenue...)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>126</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>126</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>DQC_0091</t>
+          <t>DQC_0015</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Percentage items greater than 1,000% (value &gt; 10)</t>
+          <t>Negative values for elements that cannot be negative</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>DQC_0095</t>
+          <t>DQC_0036</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Scale of cover-page shares outstanding vs balance-sheet shares</t>
+          <t>Document period end date vs the period the statements report</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>DQC_0125</t>
+          <t>DQC_0091</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Lease cost cannot be negative (unless sublease income is reported)</t>
+          <t>Percentage items greater than 1,000% (value &gt; 10)</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -726,42 +729,84 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>DQC_0194</t>
+          <t>DQC_0095</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Negative equity movements on the equity components axis</t>
+          <t>Scale of cover-page shares outstanding vs balance-sheet shares</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>DQC_0125</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Lease cost cannot be negative (unless sublease income is reported)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>DQC_0194</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Negative equity movements on the equity components axis</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>47</v>
+      </c>
+      <c r="D17" t="n">
+        <v>24</v>
+      </c>
+      <c r="E17" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>DQC_0195</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Invalid member on the equity components axis for the line item</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C18" t="n">
         <v>199</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D18" t="n">
         <v>67</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -779,6 +824,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -790,7 +837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -816,7 +863,7 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>DQC_0095: Scale of cover-page shares outstanding vs balance-sheet shares</t>
+          <t>DQC_0036: Document period end date vs the period the statements report</t>
         </is>
       </c>
     </row>
@@ -887,9 +934,194 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ELME COMMUNITIES</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>104894</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>0000104894-26-000019</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DocumentPeriodEndDate</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="5" t="n">
+        <v>46112</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" s="6" t="n">
+        <v>20250331</v>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>20260331</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>The period of report 20250331 does not match the period the statements report (20260331). Check that DocumentPeriodEndDate was updated for this filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>APARTMENT INVESTMENT &amp; MANAGEMENT CO</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>922864</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>0001193125-26-216904</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>DocumentPeriodEndDate</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" s="5" t="n">
+        <v>46112</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" s="6" t="n">
+        <v>20260131</v>
+      </c>
+      <c r="L4" s="6" t="n">
+        <v>20260331</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>The period of report 20260131 does not match the period the statements report (20260331). Check that DocumentPeriodEndDate was updated for this filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>INDONESIA ENERGY CORP LTD</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1757840</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>20-F</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>0001493152-26-019641</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DocumentPeriodEndDate</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" s="5" t="n">
+        <v>46142</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" s="6" t="n">
+        <v>20251231</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>20260430</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>The period of report 20251231 does not match the period the statements report (20260430). Check that DocumentPeriodEndDate was updated for this filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NATURALSHRIMP INC</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1465470</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>10-Q</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>0001493152-26-026574</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DocumentPeriodEndDate</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="5" t="n">
+        <v>45565</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" s="6" t="n">
+        <v>20250930</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>20240930</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>The period of report 20250930 does not match the period the statements report (20240930). Check that DocumentPeriodEndDate was updated for this filing.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A2:M6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -927,7 +1159,7 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>DQC_0125: Lease cost cannot be negative (unless sublease income is reported)</t>
+          <t>DQC_0091: Percentage items greater than 1,000% (value &gt; 10)</t>
         </is>
       </c>
     </row>
@@ -1007,6 +1239,228 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="90" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Summary</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>DQC_0095: Scale of cover-page shares outstanding vs balance-sheet shares</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Filer</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CIK</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Form</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Accession</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Statement</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Period end</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Quarters</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Reported value</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Suggested correction</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Rule message</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="90" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Summary</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>DQC_0125: Lease cost cannot be negative (unless sublease income is reported)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Filer</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CIK</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Form</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Accession</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Statement</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Period end</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Quarters</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Reported value</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Suggested correction</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Rule message</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3844,7 +4298,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18213,6 +18667,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="90" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Summary</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>DQC_0008: Reversed calculation relative to the US GAAP taxonomy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Filer</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CIK</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Form</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Accession</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Concept</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Statement</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Period end</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Quarters</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Dimensions</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Reported value</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Suggested correction</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Rule message</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -19393,7 +19958,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19504,7 +20069,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19724,7 +20289,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26890,115 +27455,4 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="90" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>&lt;&lt; Summary</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>DQC_0091: Percentage items greater than 1,000% (value &gt; 10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Filer</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>CIK</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Form</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Accession</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Concept</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Statement</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Period end</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Quarters</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Dimensions</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Reported value</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Suggested correction</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Rule message</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>